<commit_message>
feat: add Croatian Open 2026
</commit_message>
<xml_diff>
--- a/rank.xlsx
+++ b/rank.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neven/Documents/github-repos/croatian-quiz-scores/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87A9AAF1-096F-DA4D-B3BD-D78E6DF47F2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78A742A9-390B-CA48-9403-5F7E31D941A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15620" firstSheet="14" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15620" firstSheet="27" activeTab="33" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SOVA 2017" sheetId="1" r:id="rId1"/>
@@ -46,19 +46,20 @@
     <sheet name="Croatian Open 2023" sheetId="27" r:id="rId31"/>
     <sheet name="Croatian Open 2024" sheetId="28" r:id="rId32"/>
     <sheet name="Croatian Open 2025" sheetId="29" r:id="rId33"/>
-    <sheet name="WQC 2014" sheetId="30" r:id="rId34"/>
-    <sheet name="WQC 2015" sheetId="31" r:id="rId35"/>
-    <sheet name="WQC 2025" sheetId="32" r:id="rId36"/>
-    <sheet name="WQC 2026" sheetId="47" r:id="rId37"/>
-    <sheet name="WQC 2024" sheetId="33" r:id="rId38"/>
-    <sheet name="WQC 2023" sheetId="34" r:id="rId39"/>
-    <sheet name="WQC 2022" sheetId="35" r:id="rId40"/>
-    <sheet name="WQC 2021" sheetId="36" r:id="rId41"/>
-    <sheet name="WQC 2020" sheetId="37" r:id="rId42"/>
-    <sheet name="WQC 2019" sheetId="38" r:id="rId43"/>
-    <sheet name="WQC 2018" sheetId="39" r:id="rId44"/>
-    <sheet name="WQC 2017" sheetId="40" r:id="rId45"/>
-    <sheet name="WQC 2016" sheetId="41" r:id="rId46"/>
+    <sheet name="Croatian Open 2026" sheetId="49" r:id="rId34"/>
+    <sheet name="WQC 2014" sheetId="30" r:id="rId35"/>
+    <sheet name="WQC 2015" sheetId="31" r:id="rId36"/>
+    <sheet name="WQC 2025" sheetId="32" r:id="rId37"/>
+    <sheet name="WQC 2026" sheetId="47" r:id="rId38"/>
+    <sheet name="WQC 2024" sheetId="33" r:id="rId39"/>
+    <sheet name="WQC 2023" sheetId="34" r:id="rId40"/>
+    <sheet name="WQC 2022" sheetId="35" r:id="rId41"/>
+    <sheet name="WQC 2021" sheetId="36" r:id="rId42"/>
+    <sheet name="WQC 2020" sheetId="37" r:id="rId43"/>
+    <sheet name="WQC 2019" sheetId="38" r:id="rId44"/>
+    <sheet name="WQC 2018" sheetId="39" r:id="rId45"/>
+    <sheet name="WQC 2017" sheetId="40" r:id="rId46"/>
+    <sheet name="WQC 2016" sheetId="41" r:id="rId47"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -77,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4524" uniqueCount="992">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4624" uniqueCount="997">
   <si>
     <t>Krešimir Štimac</t>
   </si>
@@ -3053,6 +3054,21 @@
   </si>
   <si>
     <t>Antea Barišić Vitas</t>
+  </si>
+  <si>
+    <t>Marko Janković</t>
+  </si>
+  <si>
+    <t>Andrija Golub</t>
+  </si>
+  <si>
+    <t>Karlo Vrban</t>
+  </si>
+  <si>
+    <t>Krešimir Krpan</t>
+  </si>
+  <si>
+    <t>Bruno Klišmanić</t>
   </si>
 </sst>
 </file>
@@ -38887,6 +38903,1116 @@
 </file>
 
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC6D2654-55D0-9D47-B244-5934A60862FB}">
+  <dimension ref="A1:C100"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C2">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>158</v>
+      </c>
+      <c r="C4">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>260</v>
+      </c>
+      <c r="C5">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>130</v>
+      </c>
+      <c r="C6">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>503</v>
+      </c>
+      <c r="C7">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>295</v>
+      </c>
+      <c r="C9">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>10</v>
+      </c>
+      <c r="B10" t="s">
+        <v>342</v>
+      </c>
+      <c r="C10">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>955</v>
+      </c>
+      <c r="C11">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>140</v>
+      </c>
+      <c r="C12">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>382</v>
+      </c>
+      <c r="C13">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>15</v>
+      </c>
+      <c r="B15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>659</v>
+      </c>
+      <c r="C16">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>17</v>
+      </c>
+      <c r="B17" t="s">
+        <v>427</v>
+      </c>
+      <c r="C17">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>19</v>
+      </c>
+      <c r="B19" t="s">
+        <v>391</v>
+      </c>
+      <c r="C19">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>303</v>
+      </c>
+      <c r="C20">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>21</v>
+      </c>
+      <c r="B21" t="s">
+        <v>225</v>
+      </c>
+      <c r="C21">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>22</v>
+      </c>
+      <c r="B22" t="s">
+        <v>129</v>
+      </c>
+      <c r="C22">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>22</v>
+      </c>
+      <c r="B24" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>25</v>
+      </c>
+      <c r="B25" t="s">
+        <v>300</v>
+      </c>
+      <c r="C25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>151</v>
+      </c>
+      <c r="C26">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>27</v>
+      </c>
+      <c r="B27" t="s">
+        <v>131</v>
+      </c>
+      <c r="C27">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>28</v>
+      </c>
+      <c r="B28" t="s">
+        <v>353</v>
+      </c>
+      <c r="C28">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>51</v>
+      </c>
+      <c r="C29">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>30</v>
+      </c>
+      <c r="B30" t="s">
+        <v>189</v>
+      </c>
+      <c r="C30">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>31</v>
+      </c>
+      <c r="B31" t="s">
+        <v>647</v>
+      </c>
+      <c r="C31">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>69</v>
+      </c>
+      <c r="C32">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>31</v>
+      </c>
+      <c r="B33" t="s">
+        <v>441</v>
+      </c>
+      <c r="C33">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>31</v>
+      </c>
+      <c r="B34" t="s">
+        <v>154</v>
+      </c>
+      <c r="C34">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>31</v>
+      </c>
+      <c r="B35" t="s">
+        <v>398</v>
+      </c>
+      <c r="C35">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <v>36</v>
+      </c>
+      <c r="B36" t="s">
+        <v>432</v>
+      </c>
+      <c r="C36">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>674</v>
+      </c>
+      <c r="C37">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>36</v>
+      </c>
+      <c r="B38" t="s">
+        <v>615</v>
+      </c>
+      <c r="C38">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>36</v>
+      </c>
+      <c r="B39" t="s">
+        <v>556</v>
+      </c>
+      <c r="C39">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <v>40</v>
+      </c>
+      <c r="B40" t="s">
+        <v>237</v>
+      </c>
+      <c r="C40">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>472</v>
+      </c>
+      <c r="C41">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42">
+        <v>42</v>
+      </c>
+      <c r="B42" t="s">
+        <v>284</v>
+      </c>
+      <c r="C42">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>956</v>
+      </c>
+      <c r="C43">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>42</v>
+      </c>
+      <c r="B44" t="s">
+        <v>673</v>
+      </c>
+      <c r="C44">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <v>42</v>
+      </c>
+      <c r="B45" t="s">
+        <v>46</v>
+      </c>
+      <c r="C45">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46">
+        <v>42</v>
+      </c>
+      <c r="B46" t="s">
+        <v>489</v>
+      </c>
+      <c r="C46">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>47</v>
+      </c>
+      <c r="B47" t="s">
+        <v>306</v>
+      </c>
+      <c r="C47">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48">
+        <v>48</v>
+      </c>
+      <c r="B48" t="s">
+        <v>22</v>
+      </c>
+      <c r="C48">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
+        <v>512</v>
+      </c>
+      <c r="C49">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50">
+        <v>50</v>
+      </c>
+      <c r="B50" t="s">
+        <v>26</v>
+      </c>
+      <c r="C50">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>558</v>
+      </c>
+      <c r="C51">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52">
+        <v>50</v>
+      </c>
+      <c r="B52" t="s">
+        <v>75</v>
+      </c>
+      <c r="C52">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A53">
+        <v>53</v>
+      </c>
+      <c r="B53" t="s">
+        <v>514</v>
+      </c>
+      <c r="C53">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>218</v>
+      </c>
+      <c r="C54">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55">
+        <v>53</v>
+      </c>
+      <c r="B55" t="s">
+        <v>191</v>
+      </c>
+      <c r="C55">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56">
+        <v>56</v>
+      </c>
+      <c r="B56" t="s">
+        <v>435</v>
+      </c>
+      <c r="C56">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
+        <v>29</v>
+      </c>
+      <c r="C57">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58">
+        <v>58</v>
+      </c>
+      <c r="B58" t="s">
+        <v>280</v>
+      </c>
+      <c r="C58">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="s">
+        <v>23</v>
+      </c>
+      <c r="C59">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60">
+        <v>58</v>
+      </c>
+      <c r="B60" t="s">
+        <v>63</v>
+      </c>
+      <c r="C60">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61">
+        <v>61</v>
+      </c>
+      <c r="B61" t="s">
+        <v>15</v>
+      </c>
+      <c r="C61">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
+        <v>440</v>
+      </c>
+      <c r="C62">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63">
+        <v>61</v>
+      </c>
+      <c r="B63" t="s">
+        <v>234</v>
+      </c>
+      <c r="C63">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64">
+        <v>64</v>
+      </c>
+      <c r="B64" t="s">
+        <v>433</v>
+      </c>
+      <c r="C64">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65">
+        <v>65</v>
+      </c>
+      <c r="B65" t="s">
+        <v>559</v>
+      </c>
+      <c r="C65">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="s">
+        <v>14</v>
+      </c>
+      <c r="C66">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67">
+        <v>65</v>
+      </c>
+      <c r="B67" t="s">
+        <v>484</v>
+      </c>
+      <c r="C67">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68">
+        <v>68</v>
+      </c>
+      <c r="B68" t="s">
+        <v>992</v>
+      </c>
+      <c r="C68">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="s">
+        <v>438</v>
+      </c>
+      <c r="C69">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70">
+        <v>70</v>
+      </c>
+      <c r="B70" t="s">
+        <v>74</v>
+      </c>
+      <c r="C70">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="s">
+        <v>480</v>
+      </c>
+      <c r="C71">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72">
+        <v>72</v>
+      </c>
+      <c r="B72" t="s">
+        <v>993</v>
+      </c>
+      <c r="C72">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73">
+        <v>73</v>
+      </c>
+      <c r="B73" t="s">
+        <v>527</v>
+      </c>
+      <c r="C73">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>487</v>
+      </c>
+      <c r="C74">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A75">
+        <v>75</v>
+      </c>
+      <c r="B75" t="s">
+        <v>85</v>
+      </c>
+      <c r="C75">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A76">
+        <v>76</v>
+      </c>
+      <c r="B76" t="s">
+        <v>653</v>
+      </c>
+      <c r="C76">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="s">
+        <v>935</v>
+      </c>
+      <c r="C77">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A78">
+        <v>76</v>
+      </c>
+      <c r="B78" t="s">
+        <v>25</v>
+      </c>
+      <c r="C78">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A79">
+        <v>76</v>
+      </c>
+      <c r="B79" t="s">
+        <v>104</v>
+      </c>
+      <c r="C79">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A80">
+        <v>80</v>
+      </c>
+      <c r="B80" t="s">
+        <v>677</v>
+      </c>
+      <c r="C80">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>567</v>
+      </c>
+      <c r="C81">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A82">
+        <v>80</v>
+      </c>
+      <c r="B82" t="s">
+        <v>537</v>
+      </c>
+      <c r="C82">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A83">
+        <v>83</v>
+      </c>
+      <c r="B83" t="s">
+        <v>676</v>
+      </c>
+      <c r="C83">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="s">
+        <v>198</v>
+      </c>
+      <c r="C84">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A85">
+        <v>85</v>
+      </c>
+      <c r="B85" t="s">
+        <v>453</v>
+      </c>
+      <c r="C85">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A86">
+        <v>86</v>
+      </c>
+      <c r="B86" t="s">
+        <v>79</v>
+      </c>
+      <c r="C86">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A87">
+        <v>87</v>
+      </c>
+      <c r="B87" t="s">
+        <v>958</v>
+      </c>
+      <c r="C87">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A88">
+        <v>88</v>
+      </c>
+      <c r="B88" t="s">
+        <v>364</v>
+      </c>
+      <c r="C88">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A89">
+        <v>89</v>
+      </c>
+      <c r="B89" t="s">
+        <v>735</v>
+      </c>
+      <c r="C89">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="s">
+        <v>358</v>
+      </c>
+      <c r="C90">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A91">
+        <v>91</v>
+      </c>
+      <c r="B91" t="s">
+        <v>562</v>
+      </c>
+      <c r="C91">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A92">
+        <v>92</v>
+      </c>
+      <c r="B92" t="s">
+        <v>27</v>
+      </c>
+      <c r="C92">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="s">
+        <v>348</v>
+      </c>
+      <c r="C93">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A94">
+        <v>94</v>
+      </c>
+      <c r="B94" t="s">
+        <v>994</v>
+      </c>
+      <c r="C94">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A95">
+        <v>95</v>
+      </c>
+      <c r="B95" t="s">
+        <v>652</v>
+      </c>
+      <c r="C95">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A96">
+        <v>96</v>
+      </c>
+      <c r="B96" t="s">
+        <v>995</v>
+      </c>
+      <c r="C96">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97" t="s">
+        <v>36</v>
+      </c>
+      <c r="C97">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A98">
+        <v>98</v>
+      </c>
+      <c r="B98" t="s">
+        <v>666</v>
+      </c>
+      <c r="C98">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A99">
+        <v>99</v>
+      </c>
+      <c r="B99" t="s">
+        <v>321</v>
+      </c>
+      <c r="C99">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A100">
+        <v>100</v>
+      </c>
+      <c r="B100" t="s">
+        <v>996</v>
+      </c>
+      <c r="C100">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1D00-000000000000}">
   <dimension ref="A1:C52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -39472,7 +40598,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1E00-000000000000}">
   <dimension ref="A1:C63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -40179,7 +41305,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1F00-000000000000}">
   <dimension ref="A1:C102"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -41315,7 +42441,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48222230-6720-4C49-9F89-FD6BE3B5DBF5}">
   <dimension ref="A1:C106"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -42494,7 +43620,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2000-000000000000}">
   <dimension ref="A1:C87"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -43459,1043 +44585,6 @@
       </c>
       <c r="C87" s="3">
         <v>16</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2100-000000000000}">
-  <dimension ref="A1:C93"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="2" width="8.83203125" style="3" customWidth="1"/>
-    <col min="3" max="16384" width="8.83203125" style="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="3">
-        <v>1</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1" s="3">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="3">
-        <v>2</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="3">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="3">
-        <v>3</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="3">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="3">
-        <v>4</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="3">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="3">
-        <v>5</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>570</v>
-      </c>
-      <c r="C5" s="3">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="3">
-        <v>6</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="3">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="3">
-        <v>7</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C7" s="3">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="3">
-        <v>8</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>645</v>
-      </c>
-      <c r="C8" s="3">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="3">
-        <v>9</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="C9" s="3">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="3">
-        <v>10</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C10" s="3">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="3">
-        <v>11</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C11" s="3">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="3">
-        <v>12</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="3">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="3">
-        <v>13</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C13" s="3">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" s="3">
-        <v>14</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>342</v>
-      </c>
-      <c r="C14" s="3">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" s="3">
-        <v>15</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>389</v>
-      </c>
-      <c r="C15" s="3">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" s="3">
-        <v>16</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="C16" s="3">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="3">
-        <v>17</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>300</v>
-      </c>
-      <c r="C17" s="3">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="3">
-        <v>18</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>573</v>
-      </c>
-      <c r="C18" s="3">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="3">
-        <v>19</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="C19" s="3">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="3">
-        <v>20</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="C20" s="3">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="3">
-        <v>21</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C21" s="3">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="3">
-        <v>22</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="C22" s="3">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="3">
-        <v>23</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>759</v>
-      </c>
-      <c r="C23" s="3">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" s="3">
-        <v>24</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C24" s="3">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="3">
-        <v>25</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>391</v>
-      </c>
-      <c r="C25" s="3">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" s="3">
-        <v>26</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>353</v>
-      </c>
-      <c r="C26" s="3">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" s="3">
-        <v>27</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C27" s="3">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A28" s="3">
-        <v>28</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>506</v>
-      </c>
-      <c r="C28" s="3">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A29" s="3">
-        <v>29</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C29" s="3">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" s="3">
-        <v>30</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="C30" s="3">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" s="3">
-        <v>31</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="C31" s="3">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" s="3">
-        <v>32</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="C32" s="3">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="3">
-        <v>33</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="C33" s="3">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" s="3">
-        <v>34</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>428</v>
-      </c>
-      <c r="C34" s="3">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" s="3">
-        <v>35</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C35" s="3">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" s="3">
-        <v>36</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>722</v>
-      </c>
-      <c r="C36" s="3">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" s="3">
-        <v>37</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>614</v>
-      </c>
-      <c r="C37" s="3">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" s="3">
-        <v>38</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="C38" s="3">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" s="3">
-        <v>39</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="C39" s="3">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="3">
-        <v>40</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>305</v>
-      </c>
-      <c r="C40" s="3">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" s="3">
-        <v>41</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="C41" s="3">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A42" s="3">
-        <v>42</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>397</v>
-      </c>
-      <c r="C42" s="3">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" s="3">
-        <v>43</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>313</v>
-      </c>
-      <c r="C43" s="3">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" s="3">
-        <v>44</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C44" s="3">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A45" s="3">
-        <v>45</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>744</v>
-      </c>
-      <c r="C45" s="3">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A46" s="3">
-        <v>46</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>760</v>
-      </c>
-      <c r="C46" s="3">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A47" s="3">
-        <v>47</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>761</v>
-      </c>
-      <c r="C47" s="3">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A48" s="3">
-        <v>48</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>647</v>
-      </c>
-      <c r="C48" s="3">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A49" s="3">
-        <v>49</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="C49" s="3">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A50" s="3">
-        <v>50</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>433</v>
-      </c>
-      <c r="C50" s="3">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A51" s="3">
-        <v>51</v>
-      </c>
-      <c r="B51" s="3" t="s">
-        <v>762</v>
-      </c>
-      <c r="C51" s="3">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A52" s="3">
-        <v>52</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>763</v>
-      </c>
-      <c r="C52" s="3">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A53" s="3">
-        <v>53</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="C53" s="3">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A54" s="3">
-        <v>54</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>746</v>
-      </c>
-      <c r="C54" s="3">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A55" s="3">
-        <v>55</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>733</v>
-      </c>
-      <c r="C55" s="3">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A56" s="3">
-        <v>56</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="C56" s="3">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A57" s="3">
-        <v>57</v>
-      </c>
-      <c r="B57" s="3" t="s">
-        <v>651</v>
-      </c>
-      <c r="C57" s="3">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A58" s="3">
-        <v>58</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>714</v>
-      </c>
-      <c r="C58" s="3">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A59" s="3">
-        <v>59</v>
-      </c>
-      <c r="B59" s="3" t="s">
-        <v>729</v>
-      </c>
-      <c r="C59" s="3">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A60" s="3">
-        <v>60</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>748</v>
-      </c>
-      <c r="C60" s="3">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A61" s="3">
-        <v>61</v>
-      </c>
-      <c r="B61" s="3" t="s">
-        <v>648</v>
-      </c>
-      <c r="C61" s="3">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A62" s="3">
-        <v>62</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>720</v>
-      </c>
-      <c r="C62" s="3">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A63" s="3">
-        <v>63</v>
-      </c>
-      <c r="B63" s="3" t="s">
-        <v>346</v>
-      </c>
-      <c r="C63" s="3">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A64" s="3">
-        <v>64</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>518</v>
-      </c>
-      <c r="C64" s="3">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A65" s="3">
-        <v>65</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>764</v>
-      </c>
-      <c r="C65" s="3">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A66" s="3">
-        <v>66</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>765</v>
-      </c>
-      <c r="C66" s="3">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A67" s="3">
-        <v>67</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C67" s="3">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A68" s="3">
-        <v>68</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>658</v>
-      </c>
-      <c r="C68" s="3">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A69" s="3">
-        <v>69</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>747</v>
-      </c>
-      <c r="C69" s="3">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A70" s="3">
-        <v>70</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>586</v>
-      </c>
-      <c r="C70" s="3">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A71" s="3">
-        <v>71</v>
-      </c>
-      <c r="B71" s="3" t="s">
-        <v>592</v>
-      </c>
-      <c r="C71" s="3">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A72" s="3">
-        <v>72</v>
-      </c>
-      <c r="B72" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C72" s="3">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A73" s="3">
-        <v>73</v>
-      </c>
-      <c r="B73" s="3" t="s">
-        <v>540</v>
-      </c>
-      <c r="C73" s="3">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A74" s="3">
-        <v>74</v>
-      </c>
-      <c r="B74" s="3" t="s">
-        <v>453</v>
-      </c>
-      <c r="C74" s="3">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A75" s="3">
-        <v>75</v>
-      </c>
-      <c r="B75" s="3" t="s">
-        <v>766</v>
-      </c>
-      <c r="C75" s="3">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A76" s="3">
-        <v>76</v>
-      </c>
-      <c r="B76" s="3" t="s">
-        <v>767</v>
-      </c>
-      <c r="C76" s="3">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A77" s="3">
-        <v>77</v>
-      </c>
-      <c r="B77" s="3" t="s">
-        <v>656</v>
-      </c>
-      <c r="C77" s="3">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A78" s="3">
-        <v>78</v>
-      </c>
-      <c r="B78" s="3" t="s">
-        <v>529</v>
-      </c>
-      <c r="C78" s="3">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A79" s="3">
-        <v>79</v>
-      </c>
-      <c r="B79" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="C79" s="3">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A80" s="3">
-        <v>80</v>
-      </c>
-      <c r="B80" s="3" t="s">
-        <v>768</v>
-      </c>
-      <c r="C80" s="3">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A81" s="3">
-        <v>81</v>
-      </c>
-      <c r="B81" s="3" t="s">
-        <v>638</v>
-      </c>
-      <c r="C81" s="3">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A82" s="3">
-        <v>82</v>
-      </c>
-      <c r="B82" s="3" t="s">
-        <v>769</v>
-      </c>
-      <c r="C82" s="3">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A83" s="3">
-        <v>83</v>
-      </c>
-      <c r="B83" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="C83" s="3">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A84" s="3">
-        <v>84</v>
-      </c>
-      <c r="B84" s="3" t="s">
-        <v>593</v>
-      </c>
-      <c r="C84" s="3">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A85" s="3">
-        <v>85</v>
-      </c>
-      <c r="B85" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C85" s="3">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A86" s="3">
-        <v>86</v>
-      </c>
-      <c r="B86" s="3" t="s">
-        <v>770</v>
-      </c>
-      <c r="C86" s="3">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A87" s="3">
-        <v>87</v>
-      </c>
-      <c r="B87" s="3" t="s">
-        <v>464</v>
-      </c>
-      <c r="C87" s="3">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A88" s="3">
-        <v>88</v>
-      </c>
-      <c r="B88" s="3" t="s">
-        <v>608</v>
-      </c>
-      <c r="C88" s="3">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A89" s="3">
-        <v>89</v>
-      </c>
-      <c r="B89" s="3" t="s">
-        <v>771</v>
-      </c>
-      <c r="C89" s="3">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A90" s="3">
-        <v>90</v>
-      </c>
-      <c r="B90" s="3" t="s">
-        <v>772</v>
-      </c>
-      <c r="C90" s="3">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A91" s="3">
-        <v>91</v>
-      </c>
-      <c r="B91" s="3" t="s">
-        <v>773</v>
-      </c>
-      <c r="C91" s="3">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A92" s="3">
-        <v>92</v>
-      </c>
-      <c r="B92" s="3" t="s">
-        <v>774</v>
-      </c>
-      <c r="C92" s="3">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A93" s="3">
-        <v>93</v>
-      </c>
-      <c r="B93" s="3" t="s">
-        <v>775</v>
-      </c>
-      <c r="C93" s="3">
-        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -46718,6 +46807,1043 @@
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2100-000000000000}">
+  <dimension ref="A1:C93"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="2" width="8.83203125" style="3" customWidth="1"/>
+    <col min="3" max="16384" width="8.83203125" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="3">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="3">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="3">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="3">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="3">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="3">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="3">
+        <v>4</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="3">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="3">
+        <v>5</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C5" s="3">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="3">
+        <v>6</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="3">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="3">
+        <v>7</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="3">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
+        <v>8</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>645</v>
+      </c>
+      <c r="C8" s="3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="3">
+        <v>9</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C9" s="3">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="3">
+        <v>10</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="3">
+        <v>11</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C11" s="3">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="3">
+        <v>12</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="3">
+        <v>13</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C13" s="3">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="3">
+        <v>14</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="C14" s="3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="3">
+        <v>15</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C15" s="3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="3">
+        <v>16</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="C16" s="3">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="3">
+        <v>17</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="C17" s="3">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="3">
+        <v>18</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="C18" s="3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="3">
+        <v>19</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="C19" s="3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="3">
+        <v>20</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="C20" s="3">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="3">
+        <v>21</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C21" s="3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="3">
+        <v>22</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="C22" s="3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="3">
+        <v>23</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>759</v>
+      </c>
+      <c r="C23" s="3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="3">
+        <v>24</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="3">
+        <v>25</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="C25" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="3">
+        <v>26</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="C26" s="3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" s="3">
+        <v>27</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" s="3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="3">
+        <v>28</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="C28" s="3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" s="3">
+        <v>29</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" s="3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" s="3">
+        <v>30</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C30" s="3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" s="3">
+        <v>31</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C31" s="3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" s="3">
+        <v>32</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="C32" s="3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="3">
+        <v>33</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C33" s="3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" s="3">
+        <v>34</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="C34" s="3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" s="3">
+        <v>35</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35" s="3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" s="3">
+        <v>36</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>722</v>
+      </c>
+      <c r="C36" s="3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" s="3">
+        <v>37</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="C37" s="3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" s="3">
+        <v>38</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C38" s="3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" s="3">
+        <v>39</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="C39" s="3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" s="3">
+        <v>40</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C40" s="3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" s="3">
+        <v>41</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="C41" s="3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" s="3">
+        <v>42</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="C42" s="3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" s="3">
+        <v>43</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="C43" s="3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" s="3">
+        <v>44</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C44" s="3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" s="3">
+        <v>45</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>744</v>
+      </c>
+      <c r="C45" s="3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" s="3">
+        <v>46</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>760</v>
+      </c>
+      <c r="C46" s="3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" s="3">
+        <v>47</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="C47" s="3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" s="3">
+        <v>48</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>647</v>
+      </c>
+      <c r="C48" s="3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" s="3">
+        <v>49</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="C49" s="3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" s="3">
+        <v>50</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="C50" s="3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51" s="3">
+        <v>51</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>762</v>
+      </c>
+      <c r="C51" s="3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52" s="3">
+        <v>52</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="C52" s="3">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A53" s="3">
+        <v>53</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C53" s="3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54" s="3">
+        <v>54</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>746</v>
+      </c>
+      <c r="C54" s="3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55" s="3">
+        <v>55</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>733</v>
+      </c>
+      <c r="C55" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56" s="3">
+        <v>56</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="C56" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57" s="3">
+        <v>57</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>651</v>
+      </c>
+      <c r="C57" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58" s="3">
+        <v>58</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>714</v>
+      </c>
+      <c r="C58" s="3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59" s="3">
+        <v>59</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>729</v>
+      </c>
+      <c r="C59" s="3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60" s="3">
+        <v>60</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="C60" s="3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61" s="3">
+        <v>61</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>648</v>
+      </c>
+      <c r="C61" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" s="3">
+        <v>62</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>720</v>
+      </c>
+      <c r="C62" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63" s="3">
+        <v>63</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="C63" s="3">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64" s="3">
+        <v>64</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="C64" s="3">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65" s="3">
+        <v>65</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>764</v>
+      </c>
+      <c r="C65" s="3">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66" s="3">
+        <v>66</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>765</v>
+      </c>
+      <c r="C66" s="3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67" s="3">
+        <v>67</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C67" s="3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68" s="3">
+        <v>68</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>658</v>
+      </c>
+      <c r="C68" s="3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69" s="3">
+        <v>69</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="C69" s="3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70" s="3">
+        <v>70</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>586</v>
+      </c>
+      <c r="C70" s="3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71" s="3">
+        <v>71</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>592</v>
+      </c>
+      <c r="C71" s="3">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72" s="3">
+        <v>72</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C72" s="3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73" s="3">
+        <v>73</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>540</v>
+      </c>
+      <c r="C73" s="3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A74" s="3">
+        <v>74</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="C74" s="3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A75" s="3">
+        <v>75</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>766</v>
+      </c>
+      <c r="C75" s="3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A76" s="3">
+        <v>76</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>767</v>
+      </c>
+      <c r="C76" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A77" s="3">
+        <v>77</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>656</v>
+      </c>
+      <c r="C77" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A78" s="3">
+        <v>78</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="C78" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A79" s="3">
+        <v>79</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="C79" s="3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A80" s="3">
+        <v>80</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>768</v>
+      </c>
+      <c r="C80" s="3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A81" s="3">
+        <v>81</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>638</v>
+      </c>
+      <c r="C81" s="3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A82" s="3">
+        <v>82</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="C82" s="3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A83" s="3">
+        <v>83</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C83" s="3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A84" s="3">
+        <v>84</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>593</v>
+      </c>
+      <c r="C84" s="3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A85" s="3">
+        <v>85</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C85" s="3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A86" s="3">
+        <v>86</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>770</v>
+      </c>
+      <c r="C86" s="3">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A87" s="3">
+        <v>87</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="C87" s="3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A88" s="3">
+        <v>88</v>
+      </c>
+      <c r="B88" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="C88" s="3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A89" s="3">
+        <v>89</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>771</v>
+      </c>
+      <c r="C89" s="3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A90" s="3">
+        <v>90</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>772</v>
+      </c>
+      <c r="C90" s="3">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A91" s="3">
+        <v>91</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>773</v>
+      </c>
+      <c r="C91" s="3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A92" s="3">
+        <v>92</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>774</v>
+      </c>
+      <c r="C92" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A93" s="3">
+        <v>93</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>775</v>
+      </c>
+      <c r="C93" s="3">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2200-000000000000}">
   <dimension ref="A1:C91"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -47732,7 +48858,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2300-000000000000}">
   <dimension ref="A1:C119"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -49055,7 +50181,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2400-000000000000}">
   <dimension ref="A1:C82"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -49971,7 +51097,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2500-000000000000}">
   <dimension ref="A1:C173"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -51888,7 +53014,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2600-000000000000}">
   <dimension ref="A1:C200"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -54102,7 +55228,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2700-000000000000}">
   <dimension ref="A1:C118"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -55414,7 +56540,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2800-000000000000}">
   <dimension ref="A1:C79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>